<commit_message>
Updated daily log 25 Oct to 3 Oct
</commit_message>
<xml_diff>
--- a/D1P2636.xlsx
+++ b/D1P2636.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CAP776\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FB1DA391-BF6B-45AE-B61C-EFA43B5E978A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A71DE158-9367-4A6A-B6CD-407AB3330601}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="214" uniqueCount="64">
   <si>
     <t>My Data, My Code</t>
   </si>
@@ -216,6 +216,15 @@
   <si>
     <t>Very Unsatisfied</t>
   </si>
+  <si>
+    <t>low</t>
+  </si>
+  <si>
+    <t>Very Satisfied</t>
+  </si>
+  <si>
+    <t>Stressed</t>
+  </si>
 </sst>
 </file>
 
@@ -379,9 +388,9 @@
     <xf numFmtId="164" fontId="0" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -789,72 +798,72 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:14" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+      <c r="A1" s="19" t="s">
         <v>30</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18"/>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-      <c r="M1" s="18"/>
-      <c r="N1" s="18"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
+      <c r="K1" s="19"/>
+      <c r="L1" s="19"/>
+      <c r="M1" s="19"/>
+      <c r="N1" s="19"/>
     </row>
     <row r="2" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="6" t="s">
         <v>31</v>
       </c>
-      <c r="B2" s="19" t="s">
+      <c r="B2" s="20" t="s">
         <v>32</v>
       </c>
-      <c r="C2" s="19"/>
-      <c r="D2" s="19"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
       <c r="E2" s="6" t="s">
         <v>33</v>
       </c>
-      <c r="F2" s="19">
+      <c r="F2" s="20">
         <v>12628281</v>
       </c>
-      <c r="G2" s="19"/>
+      <c r="G2" s="20"/>
     </row>
     <row r="3" spans="1:14" ht="19.5" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="B3" s="19" t="s">
+      <c r="B3" s="20" t="s">
         <v>35</v>
       </c>
-      <c r="C3" s="19"/>
-      <c r="D3" s="19"/>
+      <c r="C3" s="20"/>
+      <c r="D3" s="20"/>
       <c r="E3" s="6" t="s">
         <v>36</v>
       </c>
-      <c r="F3" s="19"/>
-      <c r="G3" s="19"/>
+      <c r="F3" s="20"/>
+      <c r="G3" s="20"/>
     </row>
     <row r="4" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A4" s="20" t="s">
+      <c r="A4" s="18" t="s">
         <v>37</v>
       </c>
-      <c r="B4" s="20"/>
-      <c r="C4" s="20"/>
-      <c r="D4" s="20"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="18"/>
+      <c r="E4" s="18"/>
+      <c r="F4" s="18"/>
+      <c r="G4" s="18"/>
+      <c r="H4" s="18"/>
+      <c r="I4" s="18"/>
+      <c r="J4" s="18"/>
+      <c r="K4" s="18"/>
+      <c r="L4" s="18"/>
+      <c r="M4" s="18"/>
+      <c r="N4" s="18"/>
     </row>
     <row r="5" spans="1:14" ht="41.4" x14ac:dyDescent="0.3">
       <c r="A5" s="7" t="s">
@@ -2881,201 +2890,399 @@
       <c r="N50" s="16"/>
     </row>
     <row r="51" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A51" s="17"/>
-      <c r="B51" s="13"/>
-      <c r="C51" s="13"/>
-      <c r="D51" s="13"/>
-      <c r="E51" s="13"/>
-      <c r="F51" s="13"/>
-      <c r="G51" s="13"/>
-      <c r="H51" s="13"/>
-      <c r="I51" s="14" t="str">
+      <c r="A51" s="17">
+        <v>46290</v>
+      </c>
+      <c r="B51" s="13">
+        <v>400</v>
+      </c>
+      <c r="C51" s="13">
+        <v>20</v>
+      </c>
+      <c r="D51" s="13">
+        <v>50</v>
+      </c>
+      <c r="E51" s="13">
+        <v>30</v>
+      </c>
+      <c r="F51" s="13">
+        <v>250</v>
+      </c>
+      <c r="G51" s="13">
+        <v>5</v>
+      </c>
+      <c r="H51" s="13">
+        <v>300</v>
+      </c>
+      <c r="I51" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J51" s="14" t="str">
+        <v>1050</v>
+      </c>
+      <c r="J51" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K51" s="15"/>
-      <c r="L51" s="15"/>
-      <c r="M51" s="15"/>
+        <v>390</v>
+      </c>
+      <c r="K51" s="15" t="s">
+        <v>61</v>
+      </c>
+      <c r="L51" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="M51" s="15" t="s">
+        <v>54</v>
+      </c>
       <c r="N51" s="16"/>
     </row>
     <row r="52" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A52" s="17"/>
-      <c r="B52" s="13"/>
-      <c r="C52" s="13"/>
-      <c r="D52" s="13"/>
-      <c r="E52" s="13"/>
-      <c r="F52" s="13"/>
-      <c r="G52" s="13"/>
-      <c r="H52" s="13"/>
-      <c r="I52" s="14" t="str">
+      <c r="A52" s="17">
+        <v>46291</v>
+      </c>
+      <c r="B52" s="13">
+        <v>390</v>
+      </c>
+      <c r="C52" s="13">
+        <v>10</v>
+      </c>
+      <c r="D52" s="13">
+        <v>90</v>
+      </c>
+      <c r="E52" s="13">
+        <v>50</v>
+      </c>
+      <c r="F52" s="13">
+        <v>0</v>
+      </c>
+      <c r="G52" s="13">
+        <v>0</v>
+      </c>
+      <c r="H52" s="13">
+        <v>280</v>
+      </c>
+      <c r="I52" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J52" s="14" t="str">
+        <v>820</v>
+      </c>
+      <c r="J52" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K52" s="15"/>
-      <c r="L52" s="15"/>
-      <c r="M52" s="15"/>
+        <v>620</v>
+      </c>
+      <c r="K52" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="L52" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="M52" s="15" t="s">
+        <v>53</v>
+      </c>
       <c r="N52" s="16"/>
     </row>
     <row r="53" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A53" s="17"/>
-      <c r="B53" s="13"/>
-      <c r="C53" s="13"/>
-      <c r="D53" s="13"/>
-      <c r="E53" s="13"/>
-      <c r="F53" s="13"/>
-      <c r="G53" s="13"/>
-      <c r="H53" s="13"/>
-      <c r="I53" s="14" t="str">
+      <c r="A53" s="17">
+        <v>46292</v>
+      </c>
+      <c r="B53" s="13">
+        <v>410</v>
+      </c>
+      <c r="C53" s="13">
+        <v>30</v>
+      </c>
+      <c r="D53" s="13">
+        <v>0</v>
+      </c>
+      <c r="E53" s="13">
+        <v>0</v>
+      </c>
+      <c r="F53" s="13">
+        <v>0</v>
+      </c>
+      <c r="G53" s="13">
+        <v>0</v>
+      </c>
+      <c r="H53" s="13">
+        <v>400</v>
+      </c>
+      <c r="I53" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J53" s="14" t="str">
+        <v>840</v>
+      </c>
+      <c r="J53" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K53" s="15"/>
-      <c r="L53" s="15"/>
-      <c r="M53" s="15"/>
+        <v>600</v>
+      </c>
+      <c r="K53" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="L53" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="M53" s="15" t="s">
+        <v>57</v>
+      </c>
       <c r="N53" s="16"/>
     </row>
     <row r="54" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A54" s="17"/>
-      <c r="B54" s="13"/>
-      <c r="C54" s="13"/>
-      <c r="D54" s="13"/>
-      <c r="E54" s="13"/>
-      <c r="F54" s="13"/>
-      <c r="G54" s="13"/>
-      <c r="H54" s="13"/>
-      <c r="I54" s="14" t="str">
+      <c r="A54" s="17">
+        <v>46293</v>
+      </c>
+      <c r="B54" s="13">
+        <v>300</v>
+      </c>
+      <c r="C54" s="13">
+        <v>20</v>
+      </c>
+      <c r="D54" s="13">
+        <v>0</v>
+      </c>
+      <c r="E54" s="13">
+        <v>0</v>
+      </c>
+      <c r="F54" s="13">
+        <v>0</v>
+      </c>
+      <c r="G54" s="13">
+        <v>0</v>
+      </c>
+      <c r="H54" s="13">
+        <v>350</v>
+      </c>
+      <c r="I54" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J54" s="14" t="str">
+        <v>670</v>
+      </c>
+      <c r="J54" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K54" s="15"/>
-      <c r="L54" s="15"/>
-      <c r="M54" s="15"/>
+        <v>770</v>
+      </c>
+      <c r="K54" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="L54" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="M54" s="15" t="s">
+        <v>53</v>
+      </c>
       <c r="N54" s="16"/>
     </row>
     <row r="55" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A55" s="17"/>
-      <c r="B55" s="13"/>
-      <c r="C55" s="13"/>
-      <c r="D55" s="13"/>
-      <c r="E55" s="13"/>
-      <c r="F55" s="13"/>
-      <c r="G55" s="13"/>
-      <c r="H55" s="13"/>
-      <c r="I55" s="14" t="str">
+      <c r="A55" s="17">
+        <v>46294</v>
+      </c>
+      <c r="B55" s="13">
+        <v>399</v>
+      </c>
+      <c r="C55" s="13">
+        <v>20</v>
+      </c>
+      <c r="D55" s="13">
+        <v>0</v>
+      </c>
+      <c r="E55" s="13">
+        <v>0</v>
+      </c>
+      <c r="F55" s="13">
+        <v>0</v>
+      </c>
+      <c r="G55" s="13">
+        <v>0</v>
+      </c>
+      <c r="H55" s="13">
+        <v>290</v>
+      </c>
+      <c r="I55" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J55" s="14" t="str">
+        <v>709</v>
+      </c>
+      <c r="J55" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K55" s="15"/>
-      <c r="L55" s="15"/>
-      <c r="M55" s="15"/>
+        <v>731</v>
+      </c>
+      <c r="K55" s="15" t="s">
+        <v>63</v>
+      </c>
+      <c r="L55" s="15" t="s">
+        <v>56</v>
+      </c>
+      <c r="M55" s="15" t="s">
+        <v>54</v>
+      </c>
       <c r="N55" s="16"/>
     </row>
     <row r="56" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A56" s="17"/>
-      <c r="B56" s="13"/>
-      <c r="C56" s="13"/>
-      <c r="D56" s="13"/>
-      <c r="E56" s="13"/>
-      <c r="F56" s="13"/>
-      <c r="G56" s="13"/>
-      <c r="H56" s="13"/>
-      <c r="I56" s="14" t="str">
+      <c r="A56" s="17">
+        <v>46295</v>
+      </c>
+      <c r="B56" s="13">
+        <v>368</v>
+      </c>
+      <c r="C56" s="13">
+        <v>40</v>
+      </c>
+      <c r="D56" s="13">
+        <v>120</v>
+      </c>
+      <c r="E56" s="13">
+        <v>65</v>
+      </c>
+      <c r="F56" s="13">
+        <v>0</v>
+      </c>
+      <c r="G56" s="13">
+        <v>0</v>
+      </c>
+      <c r="H56" s="13">
+        <v>210</v>
+      </c>
+      <c r="I56" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J56" s="14" t="str">
+        <v>803</v>
+      </c>
+      <c r="J56" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K56" s="15"/>
-      <c r="L56" s="15"/>
-      <c r="M56" s="15"/>
+        <v>637</v>
+      </c>
+      <c r="K56" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="L56" s="15" t="s">
+        <v>52</v>
+      </c>
+      <c r="M56" s="15" t="s">
+        <v>53</v>
+      </c>
       <c r="N56" s="16"/>
     </row>
     <row r="57" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A57" s="17"/>
-      <c r="B57" s="13"/>
-      <c r="C57" s="13"/>
-      <c r="D57" s="13"/>
-      <c r="E57" s="13"/>
-      <c r="F57" s="13"/>
-      <c r="G57" s="13"/>
-      <c r="H57" s="13"/>
-      <c r="I57" s="14" t="str">
+      <c r="A57" s="17">
+        <v>46296</v>
+      </c>
+      <c r="B57" s="13">
+        <v>400</v>
+      </c>
+      <c r="C57" s="13">
+        <v>20</v>
+      </c>
+      <c r="D57" s="13">
+        <v>100</v>
+      </c>
+      <c r="E57" s="13">
+        <v>90</v>
+      </c>
+      <c r="F57" s="13">
+        <v>0</v>
+      </c>
+      <c r="G57" s="13">
+        <v>0</v>
+      </c>
+      <c r="H57" s="13">
+        <v>180</v>
+      </c>
+      <c r="I57" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J57" s="14" t="str">
+        <v>790</v>
+      </c>
+      <c r="J57" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K57" s="15"/>
-      <c r="L57" s="15"/>
-      <c r="M57" s="15"/>
+        <v>650</v>
+      </c>
+      <c r="K57" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="L57" s="15" t="s">
+        <v>58</v>
+      </c>
+      <c r="M57" s="15" t="s">
+        <v>53</v>
+      </c>
       <c r="N57" s="16"/>
     </row>
     <row r="58" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A58" s="17"/>
-      <c r="B58" s="13"/>
-      <c r="C58" s="13"/>
-      <c r="D58" s="13"/>
-      <c r="E58" s="13"/>
-      <c r="F58" s="13"/>
-      <c r="G58" s="13"/>
-      <c r="H58" s="13"/>
-      <c r="I58" s="14" t="str">
+      <c r="A58" s="17">
+        <v>46297</v>
+      </c>
+      <c r="B58" s="13">
+        <v>420</v>
+      </c>
+      <c r="C58" s="13">
+        <v>20</v>
+      </c>
+      <c r="D58" s="13">
+        <v>89</v>
+      </c>
+      <c r="E58" s="13">
+        <v>80</v>
+      </c>
+      <c r="F58" s="13">
+        <v>0</v>
+      </c>
+      <c r="G58" s="13">
+        <v>0</v>
+      </c>
+      <c r="H58" s="13">
+        <v>400</v>
+      </c>
+      <c r="I58" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J58" s="14" t="str">
+        <v>1009</v>
+      </c>
+      <c r="J58" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K58" s="15"/>
-      <c r="L58" s="15"/>
-      <c r="M58" s="15"/>
+        <v>431</v>
+      </c>
+      <c r="K58" s="15" t="s">
+        <v>55</v>
+      </c>
+      <c r="L58" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="M58" s="15" t="s">
+        <v>57</v>
+      </c>
       <c r="N58" s="16"/>
     </row>
     <row r="59" spans="1:14" x14ac:dyDescent="0.3">
-      <c r="A59" s="17"/>
-      <c r="B59" s="13"/>
-      <c r="C59" s="13"/>
-      <c r="D59" s="13"/>
-      <c r="E59" s="13"/>
-      <c r="F59" s="13"/>
-      <c r="G59" s="13"/>
-      <c r="H59" s="13"/>
-      <c r="I59" s="14" t="str">
+      <c r="A59" s="17">
+        <v>46298</v>
+      </c>
+      <c r="B59" s="13">
+        <v>350</v>
+      </c>
+      <c r="C59" s="13">
+        <v>20</v>
+      </c>
+      <c r="D59" s="13">
+        <v>90</v>
+      </c>
+      <c r="E59" s="13">
+        <v>45</v>
+      </c>
+      <c r="F59" s="13">
+        <v>0</v>
+      </c>
+      <c r="G59" s="13">
+        <v>0</v>
+      </c>
+      <c r="H59" s="13">
+        <v>350</v>
+      </c>
+      <c r="I59" s="14">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J59" s="14" t="str">
+        <v>855</v>
+      </c>
+      <c r="J59" s="14">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-      <c r="K59" s="15"/>
-      <c r="L59" s="15"/>
-      <c r="M59" s="15"/>
+        <v>585</v>
+      </c>
+      <c r="K59" s="15" t="s">
+        <v>59</v>
+      </c>
+      <c r="L59" s="15" t="s">
+        <v>62</v>
+      </c>
+      <c r="M59" s="15" t="s">
+        <v>57</v>
+      </c>
       <c r="N59" s="16"/>
     </row>
     <row r="60" spans="1:14" x14ac:dyDescent="0.3">

</xml_diff>